<commit_message>
Leads: 2026-09-24 00:12 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Innovative Roofing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>innovativeroofusa.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.innovativeroofusa.com/omaha/bellevue</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mission Take</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>info@innovativeroofusa.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(402) 512-4200</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Bellevue NE</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>88</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>roofer Bellevue NE</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 00:19 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lon Smith Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>lonsmith.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.lonsmith.com/denton-roofing/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Information Collection</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@lonsmith.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>800-317-4791</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roof replacement Denton TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 00:20 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>USA Green Air</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>usagreenairllc.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://usagreenairllc.com/hvac-contractor-brooklyn-ny/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pro Tip</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@usagreenairllc.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>347-567-8219</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HVAC contractor Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 00:24 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Miller Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>millerroofingqc.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://millerroofingqc.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Quad Cities</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>joseph@millerroofingqc.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>563-505-5179</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof replacement Davenport IA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 19:54 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A&amp;S Nathan Heating &amp; Cooling LLC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nathanheating.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://nathanheating.com/heating/repair/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Locally Trusted</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>admin@nathanheating.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(203) 735-5332</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>New Haven CT</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>furnace repair New Haven CT</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 19:59 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -863,6 +863,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ferdi Roofing and Siding</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ferdiroofingandsiding.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://ferdiroofingandsiding.com/roofing-services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@ferdiexteriors.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(425) 495-7795</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:00 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -923,6 +923,126 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Prosperity Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>prosperityroofs.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://prosperityroofs.com/roofing-round-rock-tx</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Prosperity Roofing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@indiantypefoundry.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>5128101747</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofing contractor Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RPC Restoration Inc.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rpcrestorationinc.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://rpcrestorationinc.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@rpcrestoration.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>330-573-4059</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Akron OH</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:04 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1043,182 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Carrillo Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>carrillo-roofing.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.carrillo-roofing.com/service-areas/oxnard</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Carrillo Roofing</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@carrilloroofing.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(805) 732-1233</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofing contractor Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Legacy Roofing Services</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>legacyroofing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://legacyroofing.com/roofers-near-lorain/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Legacy Roofi</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ar@legacyrfg.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>855-772-6780</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Lorain OH</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>98</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>residential roofing company Lorain OH</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Foster Roofing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>fosterroofingco.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.fosterroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@fosterroofingco.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(805) 696-2748</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roofing contractor Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:06 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1184,7 +1184,6 @@
           <t>https://www.fosterroofingco.com/</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>info@fosterroofingco.com</t>
@@ -1214,6 +1213,122 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Roof Replacement &amp; Roof Repair Salem OR | Altura Roofing</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>alturaroofingor.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://alturaroofingor.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Siding Our</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>alturaroofing0@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1971478373</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>98</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof repair company Salem OR</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Air Tech Mechanical</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>airtechok.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.airtechok.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@airtechok.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(405) 989-6314</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>heating and cooling company Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:18 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1299,7 +1299,6 @@
           <t>https://www.airtechok.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@airtechok.com</t>
@@ -1329,6 +1328,126 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Metal Roofing Company in the Pacific Northwest | Roof Replacement, Repair, &amp; Mai</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>cherryroofing.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.cherryroofing.com/roof-systems/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Copper Copper</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@cherryroofing.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(360) 823-0127</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Elite Metal Roofing | Metal Roofing in Vancouver, WA</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>elitemetalroofing.llc</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://elitemetalroofing.llc/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Elite Metal</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@elitemetalroofing.llc</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(360) 521-2248</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:20 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1453,6 +1453,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SoFlo Plumbing Co.</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>sofloplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.sofloplumbingco.com/plumber-pembroke-pines/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>service@sofloplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(954) 738-8193</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>plumbing company Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:32 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1474,7 +1474,6 @@
           <t>https://www.sofloplumbingco.com/plumber-pembroke-pines/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>service@sofloplumbingco.com</t>
@@ -1504,6 +1503,66 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Good Tidings Plumbing, Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>goodtidingscomfort.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://goodtidingscomfort.com/woodbridge-nj/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Good Tidings</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>team@goodtidingscomfort.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(732) 301-6026</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>heating and cooling company Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:37 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1568,6 +1568,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tampa Emergency Plumber</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>emergencyplumbingrepairtampa.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbingrepairtampa.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Why Tampa</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>service@tampaemergencyplumber.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(813) 219-8764</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>emergency plumber Tampa FL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:38 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1628,6 +1628,66 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Quincy Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>quincyplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://quincyplumbingpros.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Right The</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@quincyplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(617) 307-3830</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Quincy MA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>plumber Quincy MA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:40 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1688,6 +1688,66 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Plumber Thornton CO | Kitec Repiping Specialists | Just Plumbing Inc.</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>justplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://justplumbinginc.com/locations/thornton.html</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Master Plumber</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>justplumbinginc@outlook.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(303) 472-0833</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>plumber Thornton CO</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:42 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1748,6 +1748,62 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Residential Roofing in Ogden, UT</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ogdenroofers.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://ogdenroofers.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>aj@tmclife.net</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(801) 829-9651</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>residential roofing company Ogden UT</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:52 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1769,7 +1769,6 @@
           <t>https://ogdenroofers.com/residential-roofing/</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>aj@tmclife.net</t>
@@ -1799,6 +1798,174 @@
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EZ Plumbing USA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ezplumbingusa.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.ezplumbingusa.com/corona-water-heater</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>sales@ezplumbingusa.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(844) 844-2719</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Corona CA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>water heater repair Corona CA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Alpine Temperature Control</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>alpinetemp.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.alpinetemp.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>alpinetemp@gmail.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(435) 673-5746</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>88</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>HVAC contractor St George UT</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AC by JD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>acbyjd.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://acbyjd.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>acbyjd@gmail.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(435) 632-0069</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>86</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>HVAC contractor St George UT</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 20:54 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1824,7 +1824,6 @@
           <t>https://www.ezplumbingusa.com/corona-water-heater</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>sales@ezplumbingusa.com</t>
@@ -1880,7 +1879,6 @@
           <t>https://www.alpinetemp.com/</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>alpinetemp@gmail.com</t>
@@ -1936,7 +1934,6 @@
           <t>https://acbyjd.com/</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>acbyjd@gmail.com</t>
@@ -1966,6 +1963,66 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Empire Plumbing</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>empireplumbingnd.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.empireplumbingnd.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Empire Plumbing</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>empireplumbingllc@outlook.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(701) 527-1701</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bismarck ND</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>90</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>plumbing company Bismarck ND</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:03 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2028,6 +2028,62 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HM Plumbing</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>hmplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://hmplumbingservices.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>office@hmplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>316-333-9087</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>plumbing company Wichita KS</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:13 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2049,7 +2049,6 @@
           <t>https://hmplumbingservices.com/</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>office@hmplumbingservices.com</t>
@@ -2079,6 +2078,126 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HVAC in Midland, TX  | J &amp; A Refrigeration</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>jarefrigeration.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://jarefrigeration.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Free Quot</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>j.a.refrigeration.432@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1432302888</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Midland TX</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>HVAC contractor Midland TX</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Billy Black HVAC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>billyblackhvac.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://billyblackhvac.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Time President</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@indiantypefoundry.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>833-250-4822</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Midland TX</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>78</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>HVAC contractor Midland TX</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:22 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2203,6 +2203,66 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Strong Roofing</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>strongroofs.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://strongroofs.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Mississippi Gulf</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>josea@strongroofs.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>228-313-3997</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Gulfport MS</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>98</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>roofer Gulfport MS</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:25 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2263,6 +2263,122 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wichita, KS Residential Plumber Service, Commercial Plumber, Sump Pump, Water He</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>davidliesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.davidliesplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Pedestal Sump</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>melies@davidliesplumbing.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(316) 945-0117</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>plumber Wichita KS</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>WIND HVAC INC</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>windhvacinc.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://windhvacinc.com/locations/santa-ana</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>windhvac3.0@gmail.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(562) 509-5206</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>88</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>HVAC contractor Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:26 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2344,7 +2344,6 @@
           <t>https://windhvacinc.com/locations/santa-ana</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>windhvac3.0@gmail.com</t>
@@ -2374,6 +2373,62 @@
         </is>
       </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Heat Pump Repair &amp; Installation</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>prismheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.prismheatingandair.com/services/heat-pump</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>info@hvac.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>732-278-7122</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>heat pump installation Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:35 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2399,7 +2399,6 @@
           <t>https://www.prismheatingandair.com/services/heat-pump</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>info@hvac.com</t>
@@ -2429,6 +2428,62 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Black Diamond Experts</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>bdexperts.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://bdexperts.com/hvac-services/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>blackdiamond.ccr@anyhour.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(385) 446-1019</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>heat pump installation Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:42 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2454,7 +2454,6 @@
           <t>https://bdexperts.com/hvac-services/heat-pump-installation/</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>blackdiamond.ccr@anyhour.com</t>
@@ -2484,6 +2483,62 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Furnace Repair &amp; Installation Wichita, KS</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>hvacwichitaks.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.hvacwichitaks.com/wichita-residential-hvac-services/heating.asp</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>spikerheatingandair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(316) 409-6689</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>furnace repair Wichita KS</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:45 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2509,7 +2509,6 @@
           <t>https://www.hvacwichitaks.com/wichita-residential-hvac-services/heating.asp</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>spikerheatingandair@gmail.com</t>
@@ -2539,6 +2538,122 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sky Shield Roofing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>skyshieldroofers.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://skyshieldroofers.com/santa-clarita/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Popular Local</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>skyshieldroofingca@gmail.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>888-331-3460</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>100</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>roof repair company Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PrestigeRoofing Co.</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>prestigeroofingco.repair</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>http://prestigeroofingco.repair/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Santa Clarita</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>info@prestigeroofingco.repair</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>74</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roof repair company Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 21:59 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2634,7 +2634,6 @@
           <t>info@prestigeroofingco.repair</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>Santa Clarita CA</t>
@@ -2654,6 +2653,62 @@
         </is>
       </c>
       <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Precision Air Of Northern Nevada LLC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>precisionairnevada.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://precisionairnevada.com/heat-pump-installation-in-reno-nevada/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>jledkins1@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>775-481-5079</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Reno NV</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>88</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>heat pump installation Reno NV</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:00 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2679,7 +2679,6 @@
           <t>https://precisionairnevada.com/heat-pump-installation-in-reno-nevada/</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>jledkins1@yahoo.com</t>
@@ -2709,6 +2708,118 @@
         </is>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AC Installation in Danbury</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>burnettehvac.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://burnettehvac.com/locations/danbury-ct/ac-installation</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>info@burnettehvac.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(833) 597-5501</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Danbury CT</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>AC installation Danbury CT</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AC Installation in Danbury</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>windhamcountyhvac.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://windhamcountyhvac.com/locations/danbury-ct/ac-installation</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>info@windhamcountyhvac.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(844) 764-4781</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Danbury CT</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>90</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>AC installation Danbury CT</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:09 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2734,7 +2734,6 @@
           <t>https://burnettehvac.com/locations/danbury-ct/ac-installation</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>info@burnettehvac.com</t>
@@ -2790,7 +2789,6 @@
           <t>https://windhamcountyhvac.com/locations/danbury-ct/ac-installation</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>info@windhamcountyhvac.com</t>
@@ -2820,6 +2818,62 @@
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Arch Air Services</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>archairservices.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://archairservices.com/ofallon-mo/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>archairservices@gmail.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(314) 428-4328</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>air conditioning repair OFallon MO</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:13 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2844,7 +2844,6 @@
           <t>https://archairservices.com/ofallon-mo/</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>archairservices@gmail.com</t>
@@ -2874,6 +2873,122 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>roofing-contractor</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>gbargroofing.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.gbargroofing.com/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>gbargroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(936) 525-8033</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>roof replacement Conroe TX</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Certified Roofers &amp; Commercial Builders in Conroe TX | Exteriors of Texas</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>eotroofing.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.eotroofing.com/conroe-tx</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Team At</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>info@eotroofing.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>281-766-3333</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>roof replacement Conroe TX</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:18 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2899,7 +2899,6 @@
           <t>https://www.gbargroofing.com/</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>gbargroofing@gmail.com</t>
@@ -2989,6 +2988,62 @@
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Burlington Plumbers</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>plumberarchive.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.plumberarchive.com/burlington-plumbers</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Connecting Homeowners</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>hello@plumberarchive.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>76</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>plumber Burlington VT</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:26 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3024,7 +3024,6 @@
           <t>hello@plumberarchive.com</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>Burlington VT</t>
@@ -3044,6 +3043,66 @@
         </is>
       </c>
       <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Furnace Repair in Trenton</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>southernmechanicalpros.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://southernmechanicalpros.com/locations/trenton-nj/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Pros Southern</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>info@southernmechanicalpros.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(877) 401-2635</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Trenton NJ</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>furnace repair Trenton NJ</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:38 UTC (cycle 113)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3108,6 +3108,66 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>The Roofing Guys</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>618newroof.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.618newroof.com/post/roof-repair-ofallon-mo-home-needs-reliable-protection</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>At The</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>618-639-7663</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>roof replacement OFallon MO</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:39 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3168,6 +3168,66 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Knockout Plumbing, LLC</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>knockoutplumbingaz.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://knockoutplumbingaz.com/areas-we-serve/chandler/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>East Valley</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@knockoutplumbingaz.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(602) 284-5499</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Chandler AZ</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>100</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>plumbing company Chandler AZ</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:41 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3228,6 +3228,62 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Twin Ports Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>twinportsheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://twinportsheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>service@twinportsheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(218) 461-1049</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>heating and cooling company Duluth MN</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:47 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3249,7 +3249,6 @@
           <t>https://twinportsheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>service@twinportsheatingandcooling.com</t>
@@ -3279,6 +3278,66 @@
         </is>
       </c>
       <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Trusted Roofer in Sioux Falls, SD | Roof Angels</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>sioux-falls-sd.roofangels.org</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://sioux-falls-sd.roofangels.org/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Roof Angels</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@roofangels.org</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(877) 510-0035</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>80</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>roofer Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:50 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3343,6 +3343,62 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Roto Rooter of Delmarva</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>rotorooter-delmarva.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://rotorooter-delmarva.com/plumber-in-dover-delaware/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>dispatch@edsroto.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>888-337-7686</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Dover DE</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>plumber Dover DE</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:54 UTC (cycle 124)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3364,7 +3364,6 @@
           <t>https://rotorooter-delmarva.com/plumber-in-dover-delaware/</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>dispatch@edsroto.com</t>
@@ -3394,6 +3393,66 @@
         </is>
       </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Gault Electric</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>gaultelectric.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.gaultelectric.com/air-conditioning</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Virginia Peninsula</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>info@gaultelectric.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(757) 220-3300</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Newport News VA</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>AC installation Newport News VA</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 22:58 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3458,6 +3458,66 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Athens GA Roof Replacement</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>tiptonsfinetunedcarpentry.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.tiptonsfinetunedcarpentry.com/athens-ga-roof-replacement</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Jerry Tipton</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>rusty.tftc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(706) 461-2041</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>roof replacement Athens GA</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:10 UTC (cycle 135)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3518,6 +3518,66 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Citywide Express HVAC</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>citywidexpresshvac.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://citywidexpresshvac.com/locations/grand-island-ne.html</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Say About</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>dispatch@citywidexpresshvac.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(239) 268-5978</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Grand Island NE</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>air conditioning repair Grand Island NE</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:16 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3578,6 +3578,118 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Rare Breed Plumbing, Heating, and Air</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>callrarebreed.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://callrarebreed.com/plumbing/sewer-line-repair/sandy-ut/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>office@callrarebreed.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(385) 449-0144</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Sandy UT</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>100</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>sewer repair Sandy UT</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Schwanger Bros</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>schwangerbros.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://schwangerbros.com/equipment-installations/air-conditioning-installation/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>info@schwangerbros.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(717) 393-5868</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>AC installation Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:17 UTC (cycle 140)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3599,7 +3599,6 @@
           <t>https://callrarebreed.com/plumbing/sewer-line-repair/sandy-ut/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>office@callrarebreed.com</t>
@@ -3655,7 +3654,6 @@
           <t>https://schwangerbros.com/equipment-installations/air-conditioning-installation/</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>info@schwangerbros.com</t>
@@ -3685,6 +3683,62 @@
         </is>
       </c>
       <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Metal Roof - Springfield, MA - EJS Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ejsroofingexperts.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.ejsroofingexperts.com/installation-metal-roof</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ejsroofingexperts336@gmail.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(413) 388-9224</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Springfield MA</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>92</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Springfield MA</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:23 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3709,7 +3709,6 @@
           <t>https://www.ejsroofingexperts.com/installation-metal-roof</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>ejsroofingexperts336@gmail.com</t>
@@ -3739,6 +3738,66 @@
         </is>
       </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Krantz Kooling, Heating, &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>krantzcomfort.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://krantzcomfort.com/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Generators View</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>info@krantzcomfort.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(803) 672-3224</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>heating and cooling company Columbia SC</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:25 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3803,6 +3803,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Nectar Roofing</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>nectarroofing.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.nectarroofing.com/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Nectar Roofing</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>info@nectarroofing.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(913) 553-9852</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Overland Park KS</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>100</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>roof repair company Overland Park KS</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:33 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3863,6 +3863,66 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Accurate Baker Elman</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>accurateheat.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.accurateheat.com/service-area/quincy-ma/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Why Quincy</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>info@accurateheat.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(508) 507-6063</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Quincy MA</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>AC installation Quincy MA</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:41 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3923,6 +3923,62 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Rise Up Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>riseupheating.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://riseupheating.com/services/ac-repair</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>517vent@gmail.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>517-898-7706</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>air conditioning repair Lansing MI</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:42 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3944,7 +3944,6 @@
           <t>https://riseupheating.com/services/ac-repair</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>517vent@gmail.com</t>
@@ -3974,6 +3973,66 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>The Plug Plumbing</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>theplugplumbing.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://theplugplumbing.com/service-areas/sewer-line-repair-and-replacement-college-station-tx/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Final Guidance</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>info@theplugplumbing.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(833) 869-1684</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>84</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>sewer repair College Station TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:44 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4038,6 +4038,66 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Aloha Plumbing - Annapolis Plumbing Services, Repairs, Drain cleaning</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>alohaplumbingmd.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://alohaplumbingmd.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Master Plumber</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>service@alohaplumbingmd.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(410) 610-1025</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>100</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>plumbing company Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:48 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4098,6 +4098,62 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>All or Nothing Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>allornothingroofing.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://allornothingroofing.com/service-areas/missouri/lees-summit-mo/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Reviews Accredited</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>will@aonroofing.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>86</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>roofer Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:55 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4129,7 +4129,6 @@
           <t>will@aonroofing.com</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>Lees Summit MO</t>
@@ -4149,6 +4148,62 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Matt's Sewer and Drain</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>mattsseweranddrain.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://mattsseweranddrain.com/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>theresam32@live.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>402-476-6303</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:57 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4174,7 +4174,6 @@
           <t>https://mattsseweranddrain.com/</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>theresam32@live.com</t>
@@ -4204,6 +4203,62 @@
         </is>
       </c>
       <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Legacy Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>reroofcolorado.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://reroofcolorado.com/aurora-roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>sales@reroofcolorado.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(720) 541-5000</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>100</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>roof replacement Aurora CO</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-24 23:58 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-24.xlsx
+++ b/output/leads_2026-09-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4229,7 +4229,6 @@
           <t>https://reroofcolorado.com/aurora-roof-replacement/</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>sales@reroofcolorado.com</t>
@@ -4259,6 +4258,62 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Sewer Surgeon Plumbing Heating and Air</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>casewersurgeon.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://casewersurgeon.com/service-areas/santa-ana-ca/drain-cleaning-santa-ana-ca/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>info@casewersurgeon.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>8888203938</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>drain cleaning service Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>

</xml_diff>